<commit_message>
Update index and ai service
</commit_message>
<xml_diff>
--- a/pois.xlsx
+++ b/pois.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\javiv\Desktop\APP RAIDIO\raidio-backend\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EF47CA12-3294-4011-9FE2-7D8ECDC6886E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{09C36218-72D9-4365-883E-FEAD8AD7E9B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1665,7 +1665,7 @@
     <t>"cister","Desamortizción de Mendizábal","Don Pablo Muntadas Campeny", "cascadas", "jardines", "paseo", "fotografia"</t>
   </si>
   <si>
-    <t>"…", "Bar Manolo", "un restaurante muy conocido por sus raciones", "https://www.google.com/maps/place/Bernab%C3%A9u/@40.4544295,-3.6877974,17z/data=!3m1!5s0xd4228e2361e11b7:0x67f5c76cf9a0be21!4m6!3m5!1s0xd4228e23705d39f:0xa8fff6d26e2b1988!8m2!3d40.4530196!4d-3.6883748!16zL20vMDFneGx0?entry=ttu&amp;g_ep=EgoyMDI2MDMyMi4wIKXMDSoASAFQAw%3D%3D"</t>
+    <t>{"sponsorId":"bar_001","sponsorNombre":"Bar Manolo","mensaje":"Bocadillos y terraza y cocks","url":"https://www.google.com/maps/place/Bernab%C3%A9u/@40.4544295,-3.6877974,17z/data=!3m1!5s0xd4228e2361e11b7:0x67f5c76cf9a0be21!4m6!3m5!1s0xd4228e23705d39f:0xa8fff6d26e2b1988!8m2!3d40.4530196!4d-3.6883748!16zL20vMDFneGx0?entry=ttu&amp;g_ep=EgoyMDI2MDMyMi4wIKXMDSoASAFQAw%3D%3D"}</t>
   </si>
 </sst>
 </file>
@@ -2082,7 +2082,7 @@
     <col min="12" max="12" width="10.88671875" customWidth="1"/>
     <col min="13" max="13" width="23.33203125" customWidth="1"/>
     <col min="14" max="14" width="78.44140625" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="60.5546875" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="94.44140625" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="48.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>

</xml_diff>

<commit_message>
feat: añadir 14 POIs de batalla y corregir categorías
- 4 nuevos POIs: Numancia, Campo de Alarcos, Río Guadalete, Valle del Jarama
- 10 POIs existentes actualizados con categoría batallas: Covadonga,
  Roncesvalles, Calatañazor, Almansa, Ciudad Rodrigo, Badajoz,
  Vitoria-Gasteiz, Sagunto, Teruel, Medina Sidonia
- pois_db.js regenerado desde Excel (780 POIs total)

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/pois.xlsx
+++ b/pois.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="datos_POI" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MapaPOI" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="FORMULARIO" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="datos_POI" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="MapaPOI" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="FORMULARIO" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -501,7 +501,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R777"/>
+  <dimension ref="A1:R781"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -2095,7 +2095,7 @@
       </c>
       <c r="E23" s="5" t="inlineStr">
         <is>
-          <t>🏰</t>
+          <t>⚔️</t>
         </is>
       </c>
       <c r="F23" s="4" t="n">
@@ -2109,7 +2109,7 @@
       </c>
       <c r="I23" s="4" t="inlineStr">
         <is>
-          <t>"historia", "pueblo", "cultura", "ruta"</t>
+          <t>"historia", "batallas", "pueblo", "cultura", "ruta"</t>
         </is>
       </c>
       <c r="J23" s="4" t="inlineStr">
@@ -2126,14 +2126,14 @@
         </is>
       </c>
       <c r="M23" s="4" t="n">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="N23" s="4" t="n">
         <v>80</v>
       </c>
       <c r="O23" s="4" t="inlineStr">
         <is>
-          <t>"a381", "a390", "romanos", "medieval", "dulces", "mirador"</t>
+          <t>"guadalete", "reconquista", "invasion_arabe", "711"</t>
         </is>
       </c>
       <c r="P23" s="4" t="inlineStr"/>
@@ -8955,7 +8955,7 @@
       </c>
       <c r="E123" s="5" t="inlineStr">
         <is>
-          <t>🏛️</t>
+          <t>⚔️</t>
         </is>
       </c>
       <c r="F123" s="4" t="n">
@@ -8969,12 +8969,12 @@
       </c>
       <c r="I123" s="4" t="inlineStr">
         <is>
-          <t>"historia", "provincia", "capital", "cultura", "ruta"</t>
+          <t>"historia", "batallas", "guerra_civil", "provincia", "capital", "cultura", "ruta"</t>
         </is>
       </c>
       <c r="J123" s="4" t="inlineStr">
         <is>
-          <t>capital_provincia</t>
+          <t>ciudad_batalla</t>
         </is>
       </c>
       <c r="K123" s="4" t="n">
@@ -8982,18 +8982,18 @@
       </c>
       <c r="L123" s="4" t="inlineStr">
         <is>
-          <t>cultura</t>
+          <t>historia</t>
         </is>
       </c>
       <c r="M123" s="4" t="n">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="N123" s="4" t="n">
         <v>120</v>
       </c>
       <c r="O123" s="4" t="inlineStr">
         <is>
-          <t>"a23", "mudejar", "amantes", "capitalidad"</t>
+          <t>"guerra_civil", "batalla_teruel", "frente", "invierno"</t>
         </is>
       </c>
       <c r="P123" s="4" t="inlineStr"/>
@@ -11303,7 +11303,7 @@
       </c>
       <c r="E157" s="5" t="inlineStr">
         <is>
-          <t>🕍</t>
+          <t>⚔️</t>
         </is>
       </c>
       <c r="F157" s="4" t="n">
@@ -11317,12 +11317,12 @@
       </c>
       <c r="I157" s="4" t="inlineStr">
         <is>
-          <t>"historia", "santuario", "montaña"</t>
+          <t>"historia", "batallas", "reconquista", "santuario", "montaña"</t>
         </is>
       </c>
       <c r="J157" s="4" t="inlineStr">
         <is>
-          <t>santuario</t>
+          <t>campo_batalla</t>
         </is>
       </c>
       <c r="K157" s="4" t="n">
@@ -11334,14 +11334,14 @@
         </is>
       </c>
       <c r="M157" s="4" t="n">
-        <v>125</v>
+        <v>145</v>
       </c>
       <c r="N157" s="4" t="n">
         <v>60</v>
       </c>
       <c r="O157" s="4" t="inlineStr">
         <is>
-          <t>"reconquista", "santuario", "picos_de_europa"</t>
+          <t>"reconquista", "batalla", "origen_espana", "don_pelayo"</t>
         </is>
       </c>
       <c r="P157" s="4" t="inlineStr"/>
@@ -18611,7 +18611,7 @@
       </c>
       <c r="E263" s="5" t="inlineStr">
         <is>
-          <t>🏰</t>
+          <t>⚔️</t>
         </is>
       </c>
       <c r="F263" s="4" t="n">
@@ -18625,12 +18625,12 @@
       </c>
       <c r="I263" s="4" t="inlineStr">
         <is>
-          <t>"historia", "pueblo", "arquitectura", "cultura", "datosCuriosos"</t>
+          <t>"historia", "batallas", "pueblo", "arquitectura", "cultura", "datosCuriosos"</t>
         </is>
       </c>
       <c r="J263" s="4" t="inlineStr">
         <is>
-          <t>villa_historica</t>
+          <t>ciudad_batalla</t>
         </is>
       </c>
       <c r="K263" s="4" t="n">
@@ -18638,18 +18638,18 @@
       </c>
       <c r="L263" s="4" t="inlineStr">
         <is>
-          <t>cultura</t>
+          <t>historia</t>
         </is>
       </c>
       <c r="M263" s="4" t="n">
-        <v>130</v>
+        <v>138</v>
       </c>
       <c r="N263" s="4" t="n">
         <v>90</v>
       </c>
       <c r="O263" s="4" t="inlineStr">
         <is>
-          <t>"patrimonio", "casco_historico", "paseo", "arquitectura", "historia_local", "a62", "frontera", "fortificaciones"</t>
+          <t>"guerra_independencia", "asedio", "wellington", "napoleon"</t>
         </is>
       </c>
       <c r="P263" s="4" t="inlineStr"/>
@@ -21099,7 +21099,7 @@
       </c>
       <c r="E299" s="5" t="inlineStr">
         <is>
-          <t>🏰</t>
+          <t>⚔️</t>
         </is>
       </c>
       <c r="F299" s="7" t="n">
@@ -21113,12 +21113,12 @@
       </c>
       <c r="I299" s="7" t="inlineStr">
         <is>
-          <t>"historia", "pueblo", "arquitectura", "cultura", "datosCuriosos"</t>
+          <t>"historia", "batallas", "pueblo", "arquitectura", "datosCuriosos"</t>
         </is>
       </c>
       <c r="J299" s="7" t="inlineStr">
         <is>
-          <t>villa_historica</t>
+          <t>pueblo_batalla</t>
         </is>
       </c>
       <c r="K299" s="7" t="n">
@@ -21126,18 +21126,18 @@
       </c>
       <c r="L299" s="7" t="inlineStr">
         <is>
-          <t>cultura</t>
+          <t>historia</t>
         </is>
       </c>
       <c r="M299" s="7" t="n">
-        <v>120</v>
+        <v>130</v>
       </c>
       <c r="N299" s="7" t="n">
         <v>90</v>
       </c>
       <c r="O299" s="7" t="inlineStr">
         <is>
-          <t>"patrimonio", "casco_historico", "paseo", "arquitectura", "historia_local", "medieval", "sabinares"</t>
+          <t>"almanzor", "batalla", "reconquista", "leyenda"</t>
         </is>
       </c>
       <c r="P299" s="7" t="inlineStr"/>
@@ -24407,7 +24407,7 @@
       </c>
       <c r="E347" s="5" t="inlineStr">
         <is>
-          <t>🏰</t>
+          <t>⚔️</t>
         </is>
       </c>
       <c r="F347" s="4" t="n">
@@ -24421,12 +24421,12 @@
       </c>
       <c r="I347" s="4" t="inlineStr">
         <is>
-          <t>"historia", "castillo", "ciudad", "ruta"</t>
+          <t>"historia", "batallas", "castillo", "ciudad", "ruta"</t>
         </is>
       </c>
       <c r="J347" s="4" t="inlineStr">
         <is>
-          <t>ciudad_historica</t>
+          <t>ciudad_batalla</t>
         </is>
       </c>
       <c r="K347" s="4" t="n">
@@ -24434,18 +24434,18 @@
       </c>
       <c r="L347" s="4" t="inlineStr">
         <is>
-          <t>cultura</t>
+          <t>historia</t>
         </is>
       </c>
       <c r="M347" s="4" t="n">
-        <v>133</v>
+        <v>140</v>
       </c>
       <c r="N347" s="4" t="n">
         <v>100</v>
       </c>
       <c r="O347" s="4" t="inlineStr">
         <is>
-          <t>"a31", "a35", "batalla_de_almansa", "castillo", "frontera"</t>
+          <t>"guerra_sucesion", "batalla", "borbones", "austria"</t>
         </is>
       </c>
       <c r="P347" s="4" t="inlineStr"/>
@@ -36395,7 +36395,7 @@
       </c>
       <c r="E521" s="5" t="inlineStr">
         <is>
-          <t>🏰</t>
+          <t>⚔️</t>
         </is>
       </c>
       <c r="F521" s="4" t="n">
@@ -36409,12 +36409,12 @@
       </c>
       <c r="I521" s="4" t="inlineStr">
         <is>
-          <t>"historia", "ciudad", "ruta"</t>
+          <t>"historia", "batallas", "ciudad", "ruta"</t>
         </is>
       </c>
       <c r="J521" s="4" t="inlineStr">
         <is>
-          <t>ciudad_historica</t>
+          <t>ciudad_batalla</t>
         </is>
       </c>
       <c r="K521" s="4" t="n">
@@ -36426,14 +36426,14 @@
         </is>
       </c>
       <c r="M521" s="4" t="n">
-        <v>132</v>
+        <v>145</v>
       </c>
       <c r="N521" s="4" t="n">
         <v>75</v>
       </c>
       <c r="O521" s="4" t="inlineStr">
         <is>
-          <t>"ap7", "a7", "romano", "castillo"</t>
+          <t>"anibal", "asedio", "roma", "cartago", "segunda_guerra_punica"</t>
         </is>
       </c>
       <c r="P521" s="4" t="inlineStr"/>
@@ -37295,7 +37295,7 @@
       </c>
       <c r="E534" s="5" t="inlineStr">
         <is>
-          <t>🏛️</t>
+          <t>⚔️</t>
         </is>
       </c>
       <c r="F534" s="4" t="n">
@@ -37309,12 +37309,12 @@
       </c>
       <c r="I534" s="4" t="inlineStr">
         <is>
-          <t>"historia", "provincia", "capital", "frontera", "cultura"</t>
+          <t>"historia", "batallas", "provincia", "capital", "frontera", "cultura"</t>
         </is>
       </c>
       <c r="J534" s="4" t="inlineStr">
         <is>
-          <t>capital_provincia</t>
+          <t>ciudad_batalla</t>
         </is>
       </c>
       <c r="K534" s="4" t="n">
@@ -37322,18 +37322,18 @@
       </c>
       <c r="L534" s="4" t="inlineStr">
         <is>
-          <t>cultura</t>
+          <t>historia</t>
         </is>
       </c>
       <c r="M534" s="4" t="n">
-        <v>128</v>
+        <v>138</v>
       </c>
       <c r="N534" s="4" t="n">
         <v>120</v>
       </c>
       <c r="O534" s="4" t="inlineStr">
         <is>
-          <t>"frontera", "portugal", "alcazaba", "guadiana", "ciudad_amurallada"</t>
+          <t>"guerra_independencia", "asedio", "reconquista", "frontera"</t>
         </is>
       </c>
       <c r="P534" s="4" t="inlineStr"/>
@@ -45127,7 +45127,7 @@
       </c>
       <c r="E647" s="5" t="inlineStr">
         <is>
-          <t>🥾</t>
+          <t>⚔️</t>
         </is>
       </c>
       <c r="F647" s="4" t="n">
@@ -45141,12 +45141,12 @@
       </c>
       <c r="I647" s="4" t="inlineStr">
         <is>
-          <t>"montaña", "camino", "historia"</t>
+          <t>"historia", "batallas", "montaña", "camino"</t>
         </is>
       </c>
       <c r="J647" s="4" t="inlineStr">
         <is>
-          <t>puerto_historico</t>
+          <t>puerto_batalla</t>
         </is>
       </c>
       <c r="K647" s="4" t="n">
@@ -45158,14 +45158,14 @@
         </is>
       </c>
       <c r="M647" s="4" t="n">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="N647" s="4" t="n">
         <v>75</v>
       </c>
       <c r="O647" s="4" t="inlineStr">
         <is>
-          <t>"pirineo", "camino_de_santiago", "a21"</t>
+          <t>"batalla", "carlomagno", "vascos", "camino_de_santiago"</t>
         </is>
       </c>
       <c r="P647" s="4" t="inlineStr"/>
@@ -47607,7 +47607,7 @@
       </c>
       <c r="E683" s="5" t="inlineStr">
         <is>
-          <t>🏛️</t>
+          <t>⚔️</t>
         </is>
       </c>
       <c r="F683" s="4" t="n">
@@ -47621,12 +47621,12 @@
       </c>
       <c r="I683" s="4" t="inlineStr">
         <is>
-          <t>"capital", "historia", "ruta", "cultura"</t>
+          <t>"historia", "batallas", "capital", "ruta", "cultura"</t>
         </is>
       </c>
       <c r="J683" s="4" t="inlineStr">
         <is>
-          <t>capital_provincia</t>
+          <t>ciudad_batalla</t>
         </is>
       </c>
       <c r="K683" s="4" t="n">
@@ -47634,18 +47634,18 @@
       </c>
       <c r="L683" s="4" t="inlineStr">
         <is>
-          <t>cultura</t>
+          <t>historia</t>
         </is>
       </c>
       <c r="M683" s="4" t="n">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="N683" s="4" t="n">
         <v>80</v>
       </c>
       <c r="O683" s="4" t="inlineStr">
         <is>
-          <t>"a1", "ap68", "llanada_alavesa", "capital_verde", "casco_historico"</t>
+          <t>"guerra_independencia", "batalla", "napoleon", "wellington"</t>
         </is>
       </c>
       <c r="P683" s="4" t="inlineStr"/>
@@ -54071,6 +54071,266 @@
       <c r="P777" s="9" t="inlineStr"/>
       <c r="Q777" s="9" t="inlineStr"/>
       <c r="R777" s="6" t="inlineStr"/>
+    </row>
+    <row r="778">
+      <c r="A778" t="inlineStr">
+        <is>
+          <t>Castilla y León</t>
+        </is>
+      </c>
+      <c r="B778" t="inlineStr">
+        <is>
+          <t>Soria</t>
+        </is>
+      </c>
+      <c r="C778" t="inlineStr">
+        <is>
+          <t>es_so_numancia_asedio</t>
+        </is>
+      </c>
+      <c r="D778" t="inlineStr">
+        <is>
+          <t>Numancia (el asedio romano)</t>
+        </is>
+      </c>
+      <c r="E778" t="inlineStr">
+        <is>
+          <t>⚔️</t>
+        </is>
+      </c>
+      <c r="F778" t="n">
+        <v>41.8056</v>
+      </c>
+      <c r="G778" t="n">
+        <v>-2.4297</v>
+      </c>
+      <c r="H778" t="n">
+        <v>1</v>
+      </c>
+      <c r="I778" t="inlineStr">
+        <is>
+          <t>"historia", "batallas", "asedio", "romano", "datosCuriosos"</t>
+        </is>
+      </c>
+      <c r="J778" t="inlineStr">
+        <is>
+          <t>campo_batalla</t>
+        </is>
+      </c>
+      <c r="K778" t="n">
+        <v>8000</v>
+      </c>
+      <c r="L778" t="inlineStr">
+        <is>
+          <t>historia</t>
+        </is>
+      </c>
+      <c r="M778" t="n">
+        <v>165</v>
+      </c>
+      <c r="N778" t="n">
+        <v>180</v>
+      </c>
+      <c r="O778" t="inlineStr">
+        <is>
+          <t>"asedio", "numancia", "roma", "celtiberos", "resistencia"</t>
+        </is>
+      </c>
+    </row>
+    <row r="779">
+      <c r="A779" t="inlineStr">
+        <is>
+          <t>Castilla-La Mancha</t>
+        </is>
+      </c>
+      <c r="B779" t="inlineStr">
+        <is>
+          <t>Ciudad Real</t>
+        </is>
+      </c>
+      <c r="C779" t="inlineStr">
+        <is>
+          <t>es_cr_alarcos_batalla</t>
+        </is>
+      </c>
+      <c r="D779" t="inlineStr">
+        <is>
+          <t>Campo de Alarcos (batalla de 1195)</t>
+        </is>
+      </c>
+      <c r="E779" t="inlineStr">
+        <is>
+          <t>⚔️</t>
+        </is>
+      </c>
+      <c r="F779" t="n">
+        <v>38.9425</v>
+      </c>
+      <c r="G779" t="n">
+        <v>-3.9642</v>
+      </c>
+      <c r="H779" t="n">
+        <v>1</v>
+      </c>
+      <c r="I779" t="inlineStr">
+        <is>
+          <t>"historia", "batallas", "reconquista", "datosCuriosos"</t>
+        </is>
+      </c>
+      <c r="J779" t="inlineStr">
+        <is>
+          <t>campo_batalla</t>
+        </is>
+      </c>
+      <c r="K779" t="n">
+        <v>7000</v>
+      </c>
+      <c r="L779" t="inlineStr">
+        <is>
+          <t>historia</t>
+        </is>
+      </c>
+      <c r="M779" t="n">
+        <v>145</v>
+      </c>
+      <c r="N779" t="n">
+        <v>150</v>
+      </c>
+      <c r="O779" t="inlineStr">
+        <is>
+          <t>"reconquista", "almohades", "alfonso_viii", "batalla", "derrota"</t>
+        </is>
+      </c>
+    </row>
+    <row r="780">
+      <c r="A780" t="inlineStr">
+        <is>
+          <t>Andalucía</t>
+        </is>
+      </c>
+      <c r="B780" t="inlineStr">
+        <is>
+          <t>Cádiz</t>
+        </is>
+      </c>
+      <c r="C780" t="inlineStr">
+        <is>
+          <t>es_ca_guadalete_batalla</t>
+        </is>
+      </c>
+      <c r="D780" t="inlineStr">
+        <is>
+          <t>Río Guadalete (batalla de 711)</t>
+        </is>
+      </c>
+      <c r="E780" t="inlineStr">
+        <is>
+          <t>⚔️</t>
+        </is>
+      </c>
+      <c r="F780" t="n">
+        <v>36.7167</v>
+      </c>
+      <c r="G780" t="n">
+        <v>-5.9833</v>
+      </c>
+      <c r="H780" t="n">
+        <v>1</v>
+      </c>
+      <c r="I780" t="inlineStr">
+        <is>
+          <t>"historia", "batallas", "conquista", "datosCuriosos"</t>
+        </is>
+      </c>
+      <c r="J780" t="inlineStr">
+        <is>
+          <t>campo_batalla</t>
+        </is>
+      </c>
+      <c r="K780" t="n">
+        <v>9000</v>
+      </c>
+      <c r="L780" t="inlineStr">
+        <is>
+          <t>historia</t>
+        </is>
+      </c>
+      <c r="M780" t="n">
+        <v>160</v>
+      </c>
+      <c r="N780" t="n">
+        <v>180</v>
+      </c>
+      <c r="O780" t="inlineStr">
+        <is>
+          <t>"invasion_arabe", "711", "don_rodrigo", "tariq", "fin_hispania_visigoda"</t>
+        </is>
+      </c>
+    </row>
+    <row r="781">
+      <c r="A781" t="inlineStr">
+        <is>
+          <t>Comunidad de Madrid</t>
+        </is>
+      </c>
+      <c r="B781" t="inlineStr">
+        <is>
+          <t>Madrid</t>
+        </is>
+      </c>
+      <c r="C781" t="inlineStr">
+        <is>
+          <t>es_mad_jarama_batalla</t>
+        </is>
+      </c>
+      <c r="D781" t="inlineStr">
+        <is>
+          <t>Valle del Jarama (batalla de 1937)</t>
+        </is>
+      </c>
+      <c r="E781" t="inlineStr">
+        <is>
+          <t>⚔️</t>
+        </is>
+      </c>
+      <c r="F781" t="n">
+        <v>40.2564</v>
+      </c>
+      <c r="G781" t="n">
+        <v>-3.4583</v>
+      </c>
+      <c r="H781" t="n">
+        <v>1</v>
+      </c>
+      <c r="I781" t="inlineStr">
+        <is>
+          <t>"historia", "batallas", "guerra_civil", "memoria"</t>
+        </is>
+      </c>
+      <c r="J781" t="inlineStr">
+        <is>
+          <t>campo_batalla</t>
+        </is>
+      </c>
+      <c r="K781" t="n">
+        <v>8000</v>
+      </c>
+      <c r="L781" t="inlineStr">
+        <is>
+          <t>historia</t>
+        </is>
+      </c>
+      <c r="M781" t="n">
+        <v>140</v>
+      </c>
+      <c r="N781" t="n">
+        <v>150</v>
+      </c>
+      <c r="O781" t="inlineStr">
+        <is>
+          <t>"guerra_civil", "brigadas_internacionales", "frente_madrid", "batalla"</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
chore: actualización backend (8/7/26, 22:09)
</commit_message>
<xml_diff>
--- a/pois.xlsx
+++ b/pois.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/carlos/Projects/raidio-backend/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8DD50D07-F0A9-FE4B-A001-549DBAACB588}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{617FED7B-1094-3447-A86C-9DEBFCE6617D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-1100" yWindow="-18020" windowWidth="29400" windowHeight="16660" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36505,10 +36505,10 @@
         <v>4385</v>
       </c>
       <c r="H415" s="11">
-        <v>39.466700000000003</v>
+        <v>39.795200000000001</v>
       </c>
       <c r="I415" s="11">
-        <v>-3.5333000000000001</v>
+        <v>-3.4992000000000001</v>
       </c>
       <c r="J415" s="5">
         <v>1</v>

</xml_diff>

<commit_message>
chore: actualización backend (8/7/26, 22:19)
</commit_message>
<xml_diff>
--- a/pois.xlsx
+++ b/pois.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/carlos/Projects/raidio-backend/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{617FED7B-1094-3447-A86C-9DEBFCE6617D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{19620203-E162-0B4D-A350-0776460DAC90}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-1100" yWindow="-18020" windowWidth="29400" windowHeight="16660" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36505,10 +36505,10 @@
         <v>4385</v>
       </c>
       <c r="H415" s="11">
-        <v>39.795200000000001</v>
+        <v>39.794677700000001</v>
       </c>
       <c r="I415" s="11">
-        <v>-3.4992000000000001</v>
+        <v>-3.4820440000000001</v>
       </c>
       <c r="J415" s="5">
         <v>1</v>

</xml_diff>

<commit_message>
chore: actualización backend (10/7/26, 14:34)
</commit_message>
<xml_diff>
--- a/pois.xlsx
+++ b/pois.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/carlos/Projects/raidio-backend/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{19620203-E162-0B4D-A350-0776460DAC90}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{885C3B13-EC96-D04F-9243-77F9BAC65BC2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-1100" yWindow="-18020" windowWidth="29400" windowHeight="16660" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -17714,7 +17714,7 @@
         <v>421</v>
       </c>
       <c r="M70" s="6">
-        <v>16000</v>
+        <v>18000</v>
       </c>
       <c r="N70" s="23" t="s">
         <v>101</v>

</xml_diff>

<commit_message>
chore: actualización backend (10/7/26, 14:38)
</commit_message>
<xml_diff>
--- a/pois.xlsx
+++ b/pois.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/carlos/Projects/raidio-backend/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{885C3B13-EC96-D04F-9243-77F9BAC65BC2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DED65FD4-B70A-9447-999A-3B5BF1FFA140}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-1100" yWindow="-18020" windowWidth="29400" windowHeight="16660" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -17714,7 +17714,7 @@
         <v>421</v>
       </c>
       <c r="M70" s="6">
-        <v>18000</v>
+        <v>22000</v>
       </c>
       <c r="N70" s="23" t="s">
         <v>101</v>

</xml_diff>

<commit_message>
chore: actualización backend (18/7/26, 11:50)
</commit_message>
<xml_diff>
--- a/pois.xlsx
+++ b/pois.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/carlos/Projects/raidio-backend/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{41824E27-0616-B745-A331-446C7F8C6709}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{66876ABB-6483-3747-83FE-29343D7D7B95}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="16660" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -48395,7 +48395,7 @@
         <v>3381</v>
       </c>
       <c r="M633" s="6">
-        <v>8000</v>
+        <v>12000</v>
       </c>
       <c r="N633" s="23" t="s">
         <v>101</v>

</xml_diff>

<commit_message>
chore: actualización backend (18/7/26, 11:56)
</commit_message>
<xml_diff>
--- a/pois.xlsx
+++ b/pois.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/carlos/Projects/raidio-backend/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{66876ABB-6483-3747-83FE-29343D7D7B95}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9DD73F95-4E88-0C4B-A08E-B299DA78A2DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="16660" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -48395,7 +48395,7 @@
         <v>3381</v>
       </c>
       <c r="M633" s="6">
-        <v>12000</v>
+        <v>11000</v>
       </c>
       <c r="N633" s="23" t="s">
         <v>101</v>

</xml_diff>

<commit_message>
chore: actualización backend (22/7/26, 21:57)
</commit_message>
<xml_diff>
--- a/pois.xlsx
+++ b/pois.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/carlos/Projects/raidio-backend/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{304EBEFA-B427-0849-80A9-7E7F705AA0AF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B46C34B6-08B5-0548-8B22-BA13CE44CCA7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="16660" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -13907,7 +13907,7 @@
     <col min="4" max="4" width="50" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="7" bestFit="1" customWidth="1"/>
     <col min="6" max="7" width="16" customWidth="1"/>
-    <col min="8" max="8" width="11" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="22" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="11" customWidth="1"/>
     <col min="10" max="10" width="7" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="30" bestFit="1" customWidth="1"/>
@@ -29311,10 +29311,10 @@
       <c r="F283" s="9"/>
       <c r="G283" s="9"/>
       <c r="H283" s="11">
-        <v>41.2592268</v>
+        <v>4.1259408633897001</v>
       </c>
       <c r="I283" s="11">
-        <v>-3.7534036</v>
+        <v>-3.59157939542433</v>
       </c>
       <c r="J283" s="12">
         <v>2</v>
@@ -29326,7 +29326,7 @@
         <v>4384</v>
       </c>
       <c r="M283" s="13">
-        <v>2000</v>
+        <v>2500</v>
       </c>
       <c r="N283" s="16" t="s">
         <v>312</v>

</xml_diff>

<commit_message>
chore: actualización backend (22/7/26, 22:00)
</commit_message>
<xml_diff>
--- a/pois.xlsx
+++ b/pois.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/carlos/Projects/raidio-backend/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B46C34B6-08B5-0548-8B22-BA13CE44CCA7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CE198FA7-6E1C-D54D-AD94-8E982FE22033}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="16660" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -29311,7 +29311,7 @@
       <c r="F283" s="9"/>
       <c r="G283" s="9"/>
       <c r="H283" s="11">
-        <v>4.1259408633897001</v>
+        <v>41.259408633897003</v>
       </c>
       <c r="I283" s="11">
         <v>-3.59157939542433</v>

</xml_diff>